<commit_message>
Deductible updates - Updated deductible logic for spouse and family plans - Additional health care expense scenarios added to address new deductible conditions - Deductible data taken from medical-plans-at-a-glance-2026.pdf
</commit_message>
<xml_diff>
--- a/2026 NU health comparison - FAMILY.xlsx
+++ b/2026 NU health comparison - FAMILY.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d28b3282b7dd9da/Transfer/Kellogg Master/Benefits/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pbh634\Documents\GitHub\nu-health-plan-comparison\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="350" documentId="13_ncr:1_{77191DF6-FCC8-4D80-BE69-90045571E4A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDAD92C3-A1C5-462E-AA59-89AF53A1E5A4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C305C6-DFCD-4145-B4D7-BC671752D787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <author>Paul Hively</author>
   </authors>
   <commentList>
-    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -68,7 +68,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -92,7 +92,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -116,7 +116,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -140,7 +140,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="A14" authorId="0" shapeId="0" xr:uid="{ABCF2DD9-1949-49FA-854B-6B15108DC9C0}">
       <text>
         <r>
           <rPr>
@@ -160,11 +160,11 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Total health care costs in a year where the deductible is met, but the plan does not pay for any care.</t>
+Total health care costs in a year where the deductible is met for one participant, but the plan does not pay for any care.</t>
         </r>
       </text>
     </comment>
-    <comment ref="A12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="A15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -184,7 +184,79 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Total health care costs in a year where the out-of-pocket max is reached.</t>
+Total health care costs in a year where the deductible is met for both participants, but the plan does not pay for any care.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Paul Hively:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Total health care costs in a year where the out-of-pocket max is reached for one person.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A17" authorId="0" shapeId="0" xr:uid="{B1F4031B-03FC-4360-B942-BC3D2496A51E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Paul Hively:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Total health care costs in a year where the out-of-pocket max is reached for one person and the other hits the deductible.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A18" authorId="0" shapeId="0" xr:uid="{C96D3833-BB73-43C5-8708-583B8318E7BF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Paul Hively:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Total health care costs in a year where the out-of-pocket max is reached for both participants.</t>
         </r>
       </text>
     </comment>
@@ -193,14 +265,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="63">
   <si>
     <t>HMO</t>
   </si>
   <si>
-    <t>Premium</t>
-  </si>
-  <si>
     <t>Comparison</t>
   </si>
   <si>
@@ -210,19 +279,7 @@
     <t>Yearly premium</t>
   </si>
   <si>
-    <t>OOP max</t>
-  </si>
-  <si>
-    <t>Deductible</t>
-  </si>
-  <si>
     <t>No care year costs</t>
-  </si>
-  <si>
-    <t>OOP care year costs</t>
-  </si>
-  <si>
-    <t>Deductible year costs</t>
   </si>
   <si>
     <t>Arithmetic mean</t>
@@ -360,7 +417,46 @@
     <t>$2000 maximizes the NU HSA match</t>
   </si>
   <si>
-    <t>This comparison is valid for the "you + spouse + children" coverage level and assumes a shared family deductible and OOP max for each plan.</t>
+    <t>Deductible-Ind</t>
+  </si>
+  <si>
+    <t>OOP max-Ind</t>
+  </si>
+  <si>
+    <t>Deductible year costs (1 person)</t>
+  </si>
+  <si>
+    <t>Deductible year costs (2 people)</t>
+  </si>
+  <si>
+    <t>OOP care year costs (1 person)</t>
+  </si>
+  <si>
+    <t>OOP care year costs (2 people)</t>
+  </si>
+  <si>
+    <t>Deductible (Family)</t>
+  </si>
+  <si>
+    <t>Deductible (Individual)</t>
+  </si>
+  <si>
+    <t>OOP max (Family)</t>
+  </si>
+  <si>
+    <t>OOP max (Individual)</t>
+  </si>
+  <si>
+    <t>Monthly premium</t>
+  </si>
+  <si>
+    <t>Monthly HSA</t>
+  </si>
+  <si>
+    <t>Deductible (1) + OOP costs (1)</t>
+  </si>
+  <si>
+    <t>This comparison is valid for the "you + spouse" coverage level and assumes individual deductibles within the PPO and HSAe family plans.</t>
   </si>
 </sst>
 </file>
@@ -509,7 +605,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -542,6 +638,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -900,7 +997,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Calculator!$B$9</c:f>
+              <c:f>Calculator!$B$12</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -935,34 +1032,52 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Calculator!$A$10:$A$12</c:f>
+              <c:f>Calculator!$A$13:$A$18</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>No care year costs</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Deductible year costs</c:v>
+                  <c:v>Deductible year costs (1 person)</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>OOP care year costs</c:v>
+                  <c:v>Deductible year costs (2 people)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>OOP care year costs (1 person)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Deductible (1) + OOP costs (1)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>OOP care year costs (2 people)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Calculator!$B$10:$B$12</c:f>
+              <c:f>Calculator!$B$13:$B$18</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0_);[Red]\("$"#,##0\)</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>3348.6120000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>4098.6120000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>4848.6120000000001</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
+                  <c:v>6348.6120000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7098.6120000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>9348.612000000001</c:v>
                 </c:pt>
               </c:numCache>
@@ -971,7 +1086,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-EA03-47A8-862C-C2377B486F0B}"/>
+              <c16:uniqueId val="{00000000-26B2-404A-984F-BB620B18BD4D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -980,7 +1095,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Calculator!$C$9</c:f>
+              <c:f>Calculator!$C$12</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1015,27 +1130,36 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Calculator!$A$10:$A$12</c:f>
+              <c:f>Calculator!$A$13:$A$18</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>No care year costs</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Deductible year costs</c:v>
+                  <c:v>Deductible year costs (1 person)</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>OOP care year costs</c:v>
+                  <c:v>Deductible year costs (2 people)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>OOP care year costs (1 person)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Deductible (1) + OOP costs (1)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>OOP care year costs (2 people)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Calculator!$C$10:$C$12</c:f>
+              <c:f>Calculator!$C$13:$C$18</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0_);[Red]\("$"#,##0\)</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>-172.18000000000029</c:v>
                 </c:pt>
@@ -1043,6 +1167,15 @@
                   <c:v>3827.8199999999997</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>3827.8199999999997</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3827.8199999999997</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3827.8199999999997</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>7827.82</c:v>
                 </c:pt>
               </c:numCache>
@@ -1051,7 +1184,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-EA03-47A8-862C-C2377B486F0B}"/>
+              <c16:uniqueId val="{00000001-26B2-404A-984F-BB620B18BD4D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1060,7 +1193,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Calculator!$D$9</c:f>
+              <c:f>Calculator!$D$12</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1095,34 +1228,52 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Calculator!$A$10:$A$12</c:f>
+              <c:f>Calculator!$A$13:$A$18</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>No care year costs</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Deductible year costs</c:v>
+                  <c:v>Deductible year costs (1 person)</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>OOP care year costs</c:v>
+                  <c:v>Deductible year costs (2 people)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>OOP care year costs (1 person)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Deductible (1) + OOP costs (1)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>OOP care year costs (2 people)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Calculator!$D$10:$D$12</c:f>
+              <c:f>Calculator!$D$13:$D$18</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0_);[Red]\("$"#,##0\)</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>-1031.248</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>2968.752</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>6968.7520000000004</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
+                  <c:v>5968.7520000000004</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9968.7520000000004</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>12968.752</c:v>
                 </c:pt>
               </c:numCache>
@@ -1131,7 +1282,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-EA03-47A8-862C-C2377B486F0B}"/>
+              <c16:uniqueId val="{00000002-26B2-404A-984F-BB620B18BD4D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1140,7 +1291,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Calculator!$E$9</c:f>
+              <c:f>Calculator!$E$12</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1175,27 +1326,36 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Calculator!$A$10:$A$12</c:f>
+              <c:f>Calculator!$A$13:$A$18</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>No care year costs</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Deductible year costs</c:v>
+                  <c:v>Deductible year costs (1 person)</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>OOP care year costs</c:v>
+                  <c:v>Deductible year costs (2 people)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>OOP care year costs (1 person)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Deductible (1) + OOP costs (1)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>OOP care year costs (2 people)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Calculator!$E$10:$E$12</c:f>
+              <c:f>Calculator!$E$13:$E$18</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0_);[Red]\("$"#,##0\)</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>3033.0360000000001</c:v>
                 </c:pt>
@@ -1203,6 +1363,15 @@
                   <c:v>3033.0360000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>3033.0360000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4533.0360000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4533.0360000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>6033.0360000000001</c:v>
                 </c:pt>
               </c:numCache>
@@ -1211,7 +1380,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-EA03-47A8-862C-C2377B486F0B}"/>
+              <c16:uniqueId val="{00000003-26B2-404A-984F-BB620B18BD4D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1960,21 +2129,21 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2">
+        <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F6213F7-BCEA-497D-8889-BD62D81F6067}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1998,8 +2167,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:E14">
-  <autoFilter ref="A1:E14" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:E20">
+  <autoFilter ref="A1:E20" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Comparison" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="PPO" dataDxfId="45" totalsRowDxfId="44"/>
@@ -2012,37 +2181,23 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{51683AC2-BEDC-4BE5-92AD-933E7A651806}" name="Table2108915" displayName="Table2108915" ref="B14:F19" totalsRowShown="0">
-  <autoFilter ref="B14:F19" xr:uid="{51683AC2-BEDC-4BE5-92AD-933E7A651806}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{5578569F-9920-47B9-9BEC-722E9C58E221}" name="Table210119" displayName="Table210119" ref="B34:F39" totalsRowShown="0">
+  <autoFilter ref="B34:F39" xr:uid="{5578569F-9920-47B9-9BEC-722E9C58E221}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{96BAEEEF-2516-496B-8ACF-482065BB2E79}" name="Salary tier"/>
-    <tableColumn id="2" xr3:uid="{6F0470E0-90E4-4164-A37D-DF93562E43D2}" name="PPO" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{84B41708-13F2-4A2F-8CC1-72678A9F6C37}" name="HSA+" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{49F0EF58-0236-4685-BFE3-9092BAB3511E}" name="HSAe" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{F74D76C4-2D4F-416A-9D3A-07CA9BAB6B38}" name="HMO" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{7F348ACC-A2E7-492A-A6D5-8EDDBBF86386}" name="Salary tier"/>
+    <tableColumn id="2" xr3:uid="{F7315DEE-A1CC-492F-A225-94B4EB06091F}" name="PPPO" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{E52A625B-8621-4E27-986F-CC0077C4905E}" name="SPPO" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{7606D418-1D2F-4F45-9AEB-F9C02A14EFAB}" name="VPPO" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{36444FC5-C75B-4C5A-B8FA-67D3859BE2EF}" name="HMO" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="L1:P6" totalsRowShown="0">
-  <autoFilter ref="L1:P6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Salary tier"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="PPO" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="HSA+" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="HSAe" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="HMO" dataDxfId="34"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table24" displayName="Table24" ref="K8:P10" totalsRowShown="0">
-  <autoFilter ref="K8:P10" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="L9:Q14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table24" displayName="Table24" ref="K8:P12" totalsRowShown="0">
+  <autoFilter ref="K8:P12" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="L9:Q16">
     <sortCondition ref="L1:L7"/>
   </sortState>
   <tableColumns count="6">
@@ -2057,9 +2212,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="K13:P15" totalsRowShown="0" headerRowDxfId="29" headerRowBorderDxfId="28" tableBorderDxfId="27">
-  <autoFilter ref="K13:P15" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="K15:P19" totalsRowShown="0" headerRowDxfId="29" headerRowBorderDxfId="28" tableBorderDxfId="27">
+  <autoFilter ref="K15:P19" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="6">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Cap"/>
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Provider" dataDxfId="26"/>
@@ -2072,11 +2227,25 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table5" displayName="Table5" ref="I4:I11" totalsRowShown="0" headerRowDxfId="21">
   <autoFilter ref="I4:I11" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Federal Tax Brackets" dataDxfId="20"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="L1:P6" totalsRowShown="0">
+  <autoFilter ref="L1:P6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Salary tier"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="PPO" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="HSA+" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="HSAe" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="HMO" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2127,28 +2296,28 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{3C800A16-2858-4153-B93D-29BD3D5CB5E2}" name="Table21011" displayName="Table21011" ref="B34:F39" totalsRowShown="0">
-  <autoFilter ref="B34:F39" xr:uid="{3C800A16-2858-4153-B93D-29BD3D5CB5E2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E175556D-0B4B-476A-8263-ED159186E932}" name="Table21089157" displayName="Table21089157" ref="B14:F19" totalsRowShown="0">
+  <autoFilter ref="B14:F19" xr:uid="{E175556D-0B4B-476A-8263-ED159186E932}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{63FAE90E-2C65-4257-A7B0-F0640C05E29B}" name="Salary tier"/>
-    <tableColumn id="2" xr3:uid="{8E6CD055-FF43-4A10-89DC-A5292AE847B3}" name="PPPO" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{1708534C-1047-4CCA-907C-56FA034D01C5}" name="SPPO" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{F06F780A-03B0-4BC5-B914-1BCBDC39A141}" name="VPPO" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{1F0422C6-FBED-4342-9B60-2A6B7952866C}" name="HMO" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{DB793BE8-3078-4174-8915-4ED099EBD61F}" name="Salary tier"/>
+    <tableColumn id="2" xr3:uid="{9916A952-BB7C-4E53-A1AE-5210B799ACAB}" name="PPO" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{045463A7-5F51-46EF-9EA4-AC7B0B6D326C}" name="HSA+" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{484356C1-0FB3-4F55-97B9-FCFD9F79236F}" name="HSAe" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{B9C13458-99FE-4A49-AC70-DC2E4D078000}" name="HMO" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{507ECAD9-D490-49BF-8A28-BA883D9D1487}" name="Table210814" displayName="Table210814" ref="B24:F29" totalsRowShown="0">
-  <autoFilter ref="B24:F29" xr:uid="{507ECAD9-D490-49BF-8A28-BA883D9D1487}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6052B09B-C9A9-4A1D-9A1C-6A2DEAFDB748}" name="Table2108148" displayName="Table2108148" ref="B24:F29" totalsRowShown="0">
+  <autoFilter ref="B24:F29" xr:uid="{6052B09B-C9A9-4A1D-9A1C-6A2DEAFDB748}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D260E50B-D498-4602-8F0F-82D7A6670E85}" name="Salary tier"/>
-    <tableColumn id="2" xr3:uid="{326A4563-13D0-4017-B295-C469B78AE040}" name="PPPO" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{1D9CEA62-7933-4C0C-985F-B46E5A9CA795}" name="SPPO" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{B6EC9077-B315-4644-8513-2145963D87C4}" name="VPPO" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{D5E11638-2FBB-44F1-9C7B-01FCD1EB152D}" name="HMO" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{65BA179A-7E55-42A7-AF55-8CBBC9826BD3}" name="Salary tier"/>
+    <tableColumn id="2" xr3:uid="{DD60DC15-9602-45DB-9B6D-31911EA93BB1}" name="PPPO" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{01D9250F-C953-4CC0-A3B4-80887E906479}" name="SPPO" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{4F7FDEBE-684F-45B0-B0E9-DA9DA8A172CF}" name="VPPO" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{E6BA41CD-B47D-4CAD-B35A-1006F4073DBA}" name="HMO" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2417,10 +2586,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
     <col min="2" max="5" width="10" customWidth="1"/>
     <col min="7" max="8" width="20.28515625" customWidth="1"/>
     <col min="9" max="9" width="25" customWidth="1"/>
@@ -2432,40 +2601,40 @@
   <sheetData>
     <row r="1" spans="1:16" ht="30">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H1" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="9" t="s">
-        <v>25</v>
-      </c>
       <c r="L1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="N1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="O1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="P1" t="s">
         <v>0</v>
@@ -2473,7 +2642,7 @@
     </row>
     <row r="2" spans="1:16">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B2" s="3">
         <f>VLOOKUP($G$2,Table2[#All],COLUMN(),0)</f>
@@ -2492,16 +2661,16 @@
         <v>346</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="I2" s="14">
         <v>0.22</v>
       </c>
       <c r="L2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="M2" s="1">
         <v>208</v>
@@ -2518,176 +2687,170 @@
     </row>
     <row r="3" spans="1:16">
       <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3">
+        <v>60</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3">
+        <f>G6/12</f>
+        <v>166.66666666666666</v>
+      </c>
+      <c r="D3" s="3">
+        <f>G6/12</f>
+        <v>166.66666666666666</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="L3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M3" s="1">
+        <v>382</v>
+      </c>
+      <c r="N3" s="1">
+        <v>270</v>
+      </c>
+      <c r="O3" s="1">
+        <v>172</v>
+      </c>
+      <c r="P3" s="1">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
         <f>B2*12</f>
         <v>4584</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C4" s="3">
         <f>C2*12</f>
         <v>3240</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D4" s="3">
         <f>D2*12</f>
         <v>2064</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E4" s="3">
         <f>E2*12</f>
         <v>4152</v>
       </c>
-      <c r="L3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M3" s="1">
-        <v>382</v>
-      </c>
-      <c r="N3" s="1">
-        <v>270</v>
-      </c>
-      <c r="O3" s="1">
-        <v>172</v>
-      </c>
-      <c r="P3" s="1">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="11">
-        <f>-1 * B3 * ($I$2 + 4.95%)</f>
+      <c r="G4" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="L4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M4" s="1">
+        <v>647</v>
+      </c>
+      <c r="N4" s="1">
+        <v>488</v>
+      </c>
+      <c r="O4" s="1">
+        <v>387</v>
+      </c>
+      <c r="P4" s="1">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="11">
+        <f>-1 * B4 * ($I$2 + 4.95%)</f>
         <v>-1235.3880000000001</v>
       </c>
-      <c r="C4" s="11">
-        <f t="shared" ref="C4:E4" si="0">-1 * C3 * ($I$2 + 4.95%)</f>
+      <c r="C5" s="11">
+        <f t="shared" ref="C5:E5" si="0">-1 * C4 * ($I$2 + 4.95%)</f>
         <v>-873.18000000000006</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D5" s="11">
         <f t="shared" si="0"/>
         <v>-556.24800000000005</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E5" s="11">
         <f t="shared" si="0"/>
         <v>-1118.9640000000002</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="I4" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="L4" t="s">
-        <v>31</v>
-      </c>
-      <c r="M4" s="1">
-        <v>647</v>
-      </c>
-      <c r="N4" s="1">
-        <v>488</v>
-      </c>
-      <c r="O4" s="1">
-        <v>387</v>
-      </c>
-      <c r="P4" s="1">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="3">
+      <c r="G5" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="12">
+        <v>0.1</v>
+      </c>
+      <c r="L5" t="s">
+        <v>13</v>
+      </c>
+      <c r="M5" s="1">
+        <v>913</v>
+      </c>
+      <c r="N5" s="1">
+        <v>735</v>
+      </c>
+      <c r="O5" s="1">
+        <v>606</v>
+      </c>
+      <c r="P5" s="1">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="3">
         <f>-1*MIN(G6, 2000)</f>
         <v>-2000</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D6" s="3">
         <f>-1*MIN(G6, 2000)</f>
         <v>-2000</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="G5" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="I5" s="12">
-        <v>0.1</v>
-      </c>
-      <c r="L5" t="s">
-        <v>18</v>
-      </c>
-      <c r="M5" s="1">
-        <v>913</v>
-      </c>
-      <c r="N5" s="1">
-        <v>735</v>
-      </c>
-      <c r="O5" s="1">
-        <v>606</v>
-      </c>
-      <c r="P5" s="1">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="11">
+      <c r="E6" s="4"/>
+      <c r="G6" s="16">
+        <v>2000</v>
+      </c>
+      <c r="I6" s="12">
+        <v>0.12</v>
+      </c>
+      <c r="L6" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="1">
+        <v>1428</v>
+      </c>
+      <c r="N6" s="1">
+        <v>1143</v>
+      </c>
+      <c r="O6" s="1">
+        <v>967</v>
+      </c>
+      <c r="P6" s="1">
+        <v>1295</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="11">
         <f>-1 * G6 * ($I$2 + 4.95%)</f>
         <v>-539</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D7" s="11">
         <f>-1 * G6 * ($I$2 + 4.95%)</f>
         <v>-539</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="G6" s="16">
-        <v>2000</v>
-      </c>
-      <c r="I6" s="12">
-        <v>0.12</v>
-      </c>
-      <c r="L6" t="s">
-        <v>19</v>
-      </c>
-      <c r="M6" s="1">
-        <v>1428</v>
-      </c>
-      <c r="N6" s="1">
-        <v>1143</v>
-      </c>
-      <c r="O6" s="1">
-        <v>967</v>
-      </c>
-      <c r="P6" s="1">
-        <v>1295</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5">
-        <f>VLOOKUP($H$2,Table24[[#All],[Provider]:[HMO]],COLUMN(),0)</f>
-        <v>1500</v>
-      </c>
-      <c r="C7" s="5">
-        <f>VLOOKUP($H$2,Table24[[#All],[Provider]:[HMO]],COLUMN(),0)</f>
-        <v>4000</v>
-      </c>
-      <c r="D7" s="5">
-        <f>VLOOKUP($H$2,Table24[[#All],[Provider]:[HMO]],COLUMN(),0)</f>
-        <v>8000</v>
-      </c>
-      <c r="E7" s="5">
-        <f>VLOOKUP($H$2,Table24[[#All],[Provider]:[HMO]],COLUMN(),0)</f>
-        <v>0</v>
-      </c>
+      <c r="E7" s="7"/>
       <c r="G7" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="H7" s="17">
         <v>6550</v>
@@ -2698,331 +2861,523 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="B8" s="5">
-        <f>VLOOKUP($H$2,Table4[[#All],[Provider]:[HMO]],COLUMN(),0)</f>
-        <v>6000</v>
+        <f>VLOOKUP($H$2,$L$9:$P$10,COLUMN(),0)</f>
+        <v>750</v>
       </c>
       <c r="C8" s="5">
-        <f>VLOOKUP($H$2,Table4[[#All],[Provider]:[HMO]],COLUMN(),0)</f>
-        <v>8000</v>
+        <f>VLOOKUP($H$2,$L$9:$P$10,COLUMN(),0)</f>
+        <v>2000</v>
       </c>
       <c r="D8" s="5">
-        <f>VLOOKUP($H$2,Table4[[#All],[Provider]:[HMO]],COLUMN(),0)</f>
-        <v>14000</v>
+        <f>VLOOKUP($H$2,$L$9:$P$10,COLUMN(),0)</f>
+        <v>4000</v>
       </c>
       <c r="E8" s="5">
-        <f>VLOOKUP($H$2,Table4[[#All],[Provider]:[HMO]],COLUMN(),0)</f>
-        <v>3000</v>
+        <f>VLOOKUP($H$2,$L$9:$P$10,COLUMN(),0)</f>
+        <v>0</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="I8" s="12">
         <v>0.24</v>
       </c>
       <c r="K8" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="L8" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="M8" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="N8" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="O8" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="P8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:16">
-      <c r="B9" s="6" t="str">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="5">
+        <f>VLOOKUP($H$2,$L$11:$P$12,COLUMN(),0)</f>
+        <v>1500</v>
+      </c>
+      <c r="C9" s="5">
+        <f>VLOOKUP($H$2,$L$11:$P$12,COLUMN(),0)</f>
+        <v>4000</v>
+      </c>
+      <c r="D9" s="5">
+        <f>VLOOKUP($H$2,$L$11:$P$12,COLUMN(),0)</f>
+        <v>8000</v>
+      </c>
+      <c r="E9" s="5">
+        <f>VLOOKUP($H$2,$L$11:$P$12,COLUMN(),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="12">
+        <v>0.32</v>
+      </c>
+      <c r="K9" t="s">
+        <v>49</v>
+      </c>
+      <c r="L9" t="s">
+        <v>18</v>
+      </c>
+      <c r="M9" s="1">
+        <v>750</v>
+      </c>
+      <c r="N9" s="1">
+        <v>2000</v>
+      </c>
+      <c r="O9" s="1">
+        <v>4000</v>
+      </c>
+      <c r="P9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="5">
+        <f>VLOOKUP($H$2,$L$16:$P$17,COLUMN(),0)</f>
+        <v>3000</v>
+      </c>
+      <c r="C10" s="5">
+        <f>VLOOKUP($H$2,$L$16:$P$17,COLUMN(),0)</f>
+        <v>4000</v>
+      </c>
+      <c r="D10" s="5">
+        <f>VLOOKUP($H$2,$L$16:$P$17,COLUMN(),0)</f>
+        <v>7000</v>
+      </c>
+      <c r="E10" s="5">
+        <f>VLOOKUP($H$2,$L$16:$P$17,COLUMN(),0)</f>
+        <v>1500</v>
+      </c>
+      <c r="I10" s="12">
+        <v>0.35</v>
+      </c>
+      <c r="K10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L10" t="s">
+        <v>19</v>
+      </c>
+      <c r="M10" s="1">
+        <v>1500</v>
+      </c>
+      <c r="N10" s="1">
+        <v>4000</v>
+      </c>
+      <c r="O10" s="1">
+        <v>8000</v>
+      </c>
+      <c r="P10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16">
+      <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="5">
+        <f>VLOOKUP($H$2,$L$18:$P$19,COLUMN(),0)</f>
+        <v>6000</v>
+      </c>
+      <c r="C11" s="5">
+        <f>VLOOKUP($H$2,$L$18:$P$19,COLUMN(),0)</f>
+        <v>8000</v>
+      </c>
+      <c r="D11" s="5">
+        <f>VLOOKUP($H$2,$L$18:$P$19,COLUMN(),0)</f>
+        <v>14000</v>
+      </c>
+      <c r="E11" s="5">
+        <f>VLOOKUP($H$2,$L$18:$P$19,COLUMN(),0)</f>
+        <v>3000</v>
+      </c>
+      <c r="I11" s="12">
+        <v>0.37</v>
+      </c>
+      <c r="K11" t="s">
+        <v>46</v>
+      </c>
+      <c r="L11" t="s">
+        <v>18</v>
+      </c>
+      <c r="M11" s="1">
+        <v>1500</v>
+      </c>
+      <c r="N11" s="1">
+        <v>4000</v>
+      </c>
+      <c r="O11" s="1">
+        <v>8000</v>
+      </c>
+      <c r="P11" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16">
+      <c r="B12" s="6" t="str">
         <f>Table1[[#Headers],[PPO]]</f>
         <v>PPO</v>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C12" s="6" t="str">
         <f>Table1[[#Headers],[HSA+]]</f>
         <v>HSA+</v>
       </c>
-      <c r="D9" s="6" t="str">
+      <c r="D12" s="6" t="str">
         <f>Table1[[#Headers],[HSAe]]</f>
         <v>HSAe</v>
       </c>
-      <c r="E9" s="6" t="str">
+      <c r="E12" s="6" t="str">
         <f>Table1[[#Headers],[HMO]]</f>
         <v>HMO</v>
       </c>
-      <c r="I9" s="12">
-        <v>0.32</v>
-      </c>
-      <c r="K9" t="s">
-        <v>51</v>
-      </c>
-      <c r="L9" t="s">
-        <v>23</v>
-      </c>
-      <c r="M9" s="1">
-        <v>1500</v>
-      </c>
-      <c r="N9" s="1">
-        <v>4000</v>
-      </c>
-      <c r="O9" s="1">
+      <c r="K12" t="s">
+        <v>46</v>
+      </c>
+      <c r="L12" t="s">
+        <v>19</v>
+      </c>
+      <c r="M12" s="1">
+        <v>3000</v>
+      </c>
+      <c r="N12" s="1">
         <v>8000</v>
       </c>
-      <c r="P9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16">
-      <c r="A10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="3">
-        <f>SUM(B3:B6)</f>
+      <c r="O12" s="1">
+        <v>16000</v>
+      </c>
+      <c r="P12" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="3">
+        <f>SUM(B4:B7)</f>
         <v>3348.6120000000001</v>
       </c>
-      <c r="C10" s="3">
-        <f>SUM(C3:C6)</f>
+      <c r="C13" s="3">
+        <f>SUM(C4:C7)</f>
         <v>-172.18000000000029</v>
       </c>
-      <c r="D10" s="3">
-        <f>SUM(D3:D6)</f>
+      <c r="D13" s="3">
+        <f>SUM(D4:D7)</f>
         <v>-1031.248</v>
       </c>
-      <c r="E10" s="3">
-        <f>SUM(E3:E6)</f>
+      <c r="E13" s="3">
+        <f>SUM(E4:E7)</f>
         <v>3033.0360000000001</v>
       </c>
-      <c r="I10" s="12">
-        <v>0.35</v>
-      </c>
-      <c r="K10" t="s">
-        <v>51</v>
-      </c>
-      <c r="L10" t="s">
-        <v>24</v>
-      </c>
-      <c r="M10" s="1">
-        <v>3000</v>
-      </c>
-      <c r="N10" s="1">
-        <v>8000</v>
-      </c>
-      <c r="O10" s="1">
-        <v>16000</v>
-      </c>
-      <c r="P10" s="1" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="3">
-        <f>SUM(B3:B7)</f>
-        <v>4848.6120000000001</v>
-      </c>
-      <c r="C11" s="3">
-        <f>SUM(C3:C7)</f>
-        <v>3827.8199999999997</v>
-      </c>
-      <c r="D11" s="3">
-        <f>SUM(D3:D7)</f>
-        <v>6968.7520000000004</v>
-      </c>
-      <c r="E11" s="3">
-        <f>SUM(E3:E7)</f>
-        <v>3033.0360000000001</v>
-      </c>
-      <c r="I11" s="12">
-        <v>0.37</v>
-      </c>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
-    </row>
-    <row r="12" spans="1:16">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="3">
-        <f>SUM(B3:B6,B8)</f>
-        <v>9348.612000000001</v>
-      </c>
-      <c r="C12" s="3">
-        <f>SUM(C3:C6,C8)</f>
-        <v>7827.82</v>
-      </c>
-      <c r="D12" s="3">
-        <f>SUM(D3:D6,D8)</f>
-        <v>12968.752</v>
-      </c>
-      <c r="E12" s="3">
-        <f>SUM(E3:E6,E8)</f>
-        <v>6033.0360000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16">
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="K13" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L13" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M13" t="s">
-        <v>39</v>
-      </c>
-      <c r="N13" t="s">
-        <v>48</v>
-      </c>
-      <c r="O13" t="s">
-        <v>49</v>
-      </c>
-      <c r="P13" t="s">
-        <v>0</v>
-      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="B14" s="3">
-        <f>AVERAGE(B10:B12)</f>
-        <v>5848.612000000001</v>
+        <f>SUM(B4:B8)</f>
+        <v>4098.6120000000001</v>
       </c>
       <c r="C14" s="3">
-        <f>AVERAGE(C10:C12)</f>
+        <f>SUM(C4:C7,C9)</f>
         <v>3827.8199999999997</v>
       </c>
       <c r="D14" s="3">
-        <f>AVERAGE(D10:D12)</f>
-        <v>6302.0853333333334</v>
+        <f>SUM(D4:D8)</f>
+        <v>2968.752</v>
       </c>
       <c r="E14" s="3">
-        <f>AVERAGE(E10:E12)</f>
-        <v>4033.0360000000001</v>
+        <f>SUM(E4:E8)</f>
+        <v>3033.0360000000001</v>
       </c>
       <c r="J14" s="2"/>
-      <c r="K14" t="s">
+    </row>
+    <row r="15" spans="1:16" ht="15" customHeight="1">
+      <c r="A15" t="s">
         <v>52</v>
       </c>
-      <c r="L14" t="s">
-        <v>23</v>
-      </c>
-      <c r="M14" s="1">
-        <v>6000</v>
-      </c>
-      <c r="N14" s="1">
-        <v>8000</v>
-      </c>
-      <c r="O14" s="1">
-        <v>14000</v>
-      </c>
-      <c r="P14" s="1">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="15" customHeight="1">
-      <c r="A15" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="B15" s="3">
+        <f>SUM(B4:B7) + MIN(B8*2,B9)</f>
+        <v>4848.6120000000001</v>
+      </c>
+      <c r="C15" s="3">
+        <f>SUM(C4:C7) + MIN(C8*2,C9)</f>
+        <v>3827.8199999999997</v>
+      </c>
+      <c r="D15" s="3">
+        <f>SUM(D4:D7) + MIN(D8*2,D9)</f>
+        <v>6968.7520000000004</v>
+      </c>
+      <c r="E15" s="3">
+        <f>SUM(E4:E7) + MIN(E8*2,E9)</f>
+        <v>3033.0360000000001</v>
+      </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" t="s">
-        <v>52</v>
-      </c>
-      <c r="L15" t="s">
-        <v>24</v>
-      </c>
-      <c r="M15" s="1">
+      <c r="K15" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="L15" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="M15" t="s">
+        <v>34</v>
+      </c>
+      <c r="N15" t="s">
+        <v>43</v>
+      </c>
+      <c r="O15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P15" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="3">
+        <f>SUM(B4:B7,B10)</f>
+        <v>6348.6120000000001</v>
+      </c>
+      <c r="C16" s="3">
+        <f>SUM(C4:C7,C10)</f>
+        <v>3827.8199999999997</v>
+      </c>
+      <c r="D16" s="3">
+        <f>SUM(D4:D7,D10)</f>
+        <v>5968.7520000000004</v>
+      </c>
+      <c r="E16" s="3">
+        <f>SUM(E4:E7,E10)</f>
+        <v>4533.0360000000001</v>
+      </c>
+      <c r="K16" t="s">
+        <v>50</v>
+      </c>
+      <c r="L16" t="s">
+        <v>18</v>
+      </c>
+      <c r="M16" s="1">
+        <v>3000</v>
+      </c>
+      <c r="N16" s="1">
+        <v>4000</v>
+      </c>
+      <c r="O16" s="1">
+        <v>7000</v>
+      </c>
+      <c r="P16" s="1">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16">
+      <c r="A17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="3">
+        <f>SUM(B4:B7)+MIN(SUM(B8,B10),B11)</f>
+        <v>7098.6120000000001</v>
+      </c>
+      <c r="C17" s="3">
+        <f>SUM(C4:C7)+MIN(IF(C10&gt;=C9,C10,C9),C11)</f>
+        <v>3827.8199999999997</v>
+      </c>
+      <c r="D17" s="3">
+        <f>SUM(D4:D7)+MIN(SUM(D8,D10),D11)</f>
+        <v>9968.7520000000004</v>
+      </c>
+      <c r="E17" s="3">
+        <f>SUM(E4:E7)+MIN(SUM(E8,E10),E11)</f>
+        <v>4533.0360000000001</v>
+      </c>
+      <c r="K17" t="s">
+        <v>50</v>
+      </c>
+      <c r="L17" t="s">
+        <v>19</v>
+      </c>
+      <c r="M17" s="1">
+        <v>6000</v>
+      </c>
+      <c r="N17" s="1">
+        <v>8000</v>
+      </c>
+      <c r="O17" s="1">
+        <v>14000</v>
+      </c>
+      <c r="P17" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="3">
+        <f>SUM(B4:B7,B11)</f>
+        <v>9348.612000000001</v>
+      </c>
+      <c r="C18" s="3">
+        <f>SUM(C4:C7,C11)</f>
+        <v>7827.82</v>
+      </c>
+      <c r="D18" s="3">
+        <f>SUM(D4:D7,D11)</f>
+        <v>12968.752</v>
+      </c>
+      <c r="E18" s="3">
+        <f>SUM(E4:E7,E11)</f>
+        <v>6033.0360000000001</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="K18" t="s">
+        <v>47</v>
+      </c>
+      <c r="L18" t="s">
+        <v>18</v>
+      </c>
+      <c r="M18" s="1">
+        <v>6000</v>
+      </c>
+      <c r="N18" s="1">
+        <v>8000</v>
+      </c>
+      <c r="O18" s="1">
+        <v>14000</v>
+      </c>
+      <c r="P18" s="1">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16">
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="K19" t="s">
+        <v>47</v>
+      </c>
+      <c r="L19" t="s">
+        <v>19</v>
+      </c>
+      <c r="M19" s="1">
         <v>12000</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N19" s="1">
         <v>16000</v>
       </c>
-      <c r="O15" s="1">
+      <c r="O19" s="1">
         <v>28000</v>
       </c>
-      <c r="P15" s="1" t="e">
+      <c r="P19" s="1" t="e">
         <v>#N/A</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
-      <c r="A16" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="2"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
+    <row r="20" spans="1:16">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="3">
+        <f>AVERAGE(B13:B18)</f>
+        <v>5848.612000000001</v>
+      </c>
+      <c r="C20" s="3">
+        <f>AVERAGE(C13:C18)</f>
+        <v>3827.8199999999997</v>
+      </c>
+      <c r="D20" s="3">
+        <f>AVERAGE(D13:D18)</f>
+        <v>6302.0853333333334</v>
+      </c>
+      <c r="E20" s="3">
+        <f>AVERAGE(E13:E18)</f>
+        <v>4033.0360000000001</v>
+      </c>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+    </row>
+    <row r="21" spans="1:16">
+      <c r="A21" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+    </row>
+    <row r="22" spans="1:16">
+      <c r="A22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+    </row>
+    <row r="23" spans="1:16">
+      <c r="A23" s="2"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+    </row>
+    <row r="24" spans="1:16">
+      <c r="A24" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+    </row>
+    <row r="25" spans="1:16">
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+    </row>
+    <row r="26" spans="1:16">
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+    </row>
+    <row r="27" spans="1:16">
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B10:E10">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B11:E11">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B12:E12">
-    <cfRule type="colorScale" priority="5">
+  <conditionalFormatting sqref="B13:E13">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3045,6 +3400,78 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E15">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:E16">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B17:E17">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18:E18">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19:E19">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B20:E20">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$L$2:$L$6</formula1>
@@ -3057,11 +3484,14 @@
       <formula2>H7</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{00000000-0002-0000-0000-000001000000}">
-      <formula1>$L$9:$L$10</formula1>
+      <formula1>$L$9:$L$12</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="C14 C17" formula="1"/>
+  </ignoredErrors>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
   <tableParts count="5">
@@ -3089,44 +3519,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="B1" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
     </row>
     <row r="4" spans="1:6">
       <c r="B4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" t="s">
         <v>45</v>
       </c>
-      <c r="D4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" t="s">
-        <v>50</v>
-      </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="21" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C5" s="18">
         <f t="shared" ref="C5:C9" si="0">C15/D25-1</f>
@@ -3147,10 +3577,10 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="21" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C6" s="18">
         <f t="shared" si="0"/>
@@ -3171,10 +3601,10 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="21" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C7" s="18">
         <f t="shared" si="0"/>
@@ -3195,10 +3625,10 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="21" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C8" s="18">
         <f t="shared" si="0"/>
@@ -3219,10 +3649,10 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="21" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C9" s="18">
         <f t="shared" si="0"/>
@@ -3242,33 +3672,33 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="B11" s="22">
+      <c r="B11" s="23">
         <v>2026</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1">
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
     </row>
     <row r="14" spans="1:6">
       <c r="B14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E14" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F14" t="s">
         <v>0</v>
@@ -3280,7 +3710,7 @@
         <v>2026A</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C15" s="1">
         <v>208</v>
@@ -3301,7 +3731,7 @@
         <v>2026B</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C16" s="1">
         <v>382</v>
@@ -3322,7 +3752,7 @@
         <v>2026C</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C17" s="1">
         <v>647</v>
@@ -3343,7 +3773,7 @@
         <v>2026D</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C18" s="1">
         <v>913</v>
@@ -3364,7 +3794,7 @@
         <v>2026E</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C19" s="1">
         <v>1428</v>
@@ -3380,40 +3810,40 @@
       </c>
     </row>
     <row r="21" spans="1:15" ht="15" customHeight="1">
-      <c r="B21" s="22">
+      <c r="B21" s="23">
         <v>2025</v>
       </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="I21" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="I21" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="23"/>
+      <c r="M21" s="23"/>
       <c r="N21" s="20" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="O21" s="10">
         <v>2025</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15" customHeight="1">
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23"/>
+      <c r="L22" s="23"/>
+      <c r="M22" s="23"/>
       <c r="N22" s="20" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="O22" s="10">
         <v>2024</v>
@@ -3421,31 +3851,31 @@
     </row>
     <row r="24" spans="1:15">
       <c r="B24" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E24" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F24" t="s">
         <v>0</v>
       </c>
       <c r="I24" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J24" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="K24" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="L24" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M24" t="s">
         <v>0</v>
@@ -3457,7 +3887,7 @@
         <v>2025A</v>
       </c>
       <c r="B25" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C25" s="1">
         <v>995</v>
@@ -3472,10 +3902,10 @@
         <v>415</v>
       </c>
       <c r="H25" s="21" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="I25" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="J25" s="18">
         <f t="shared" ref="J25:M29" si="4">VLOOKUP(Year1&amp;$A5,$A$10:$F$1019,COLUMN(C$4),0)/VLOOKUP(Year2&amp;$A5,$A$10:$F$1019,COLUMN(C$4),0)-1</f>
@@ -3500,7 +3930,7 @@
         <v>2025B</v>
       </c>
       <c r="B26" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C26" s="1">
         <v>1186</v>
@@ -3515,10 +3945,10 @@
         <v>542</v>
       </c>
       <c r="H26" s="21" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="I26" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J26" s="18">
         <f t="shared" si="4"/>
@@ -3543,7 +3973,7 @@
         <v>2025C</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C27" s="1">
         <v>1430</v>
@@ -3558,10 +3988,10 @@
         <v>706</v>
       </c>
       <c r="H27" s="21" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="I27" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="J27" s="18">
         <f t="shared" si="4"/>
@@ -3586,7 +4016,7 @@
         <v>2025D</v>
       </c>
       <c r="B28" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C28" s="1">
         <v>1751</v>
@@ -3601,10 +4031,10 @@
         <v>897</v>
       </c>
       <c r="H28" s="21" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="I28" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J28" s="18">
         <f t="shared" si="4"/>
@@ -3629,7 +4059,7 @@
         <v>2025E</v>
       </c>
       <c r="B29" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C29" s="1">
         <v>2210</v>
@@ -3644,10 +4074,10 @@
         <v>1201</v>
       </c>
       <c r="H29" s="21" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="I29" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J29" s="18">
         <f t="shared" si="4"/>
@@ -3667,34 +4097,34 @@
       </c>
     </row>
     <row r="31" spans="1:15" ht="15" customHeight="1">
-      <c r="B31" s="22">
+      <c r="B31" s="23">
         <v>2024</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
     </row>
     <row r="32" spans="1:15" ht="15" customHeight="1">
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
       <c r="H32" s="19"/>
     </row>
     <row r="34" spans="1:6">
       <c r="B34" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E34" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F34" t="s">
         <v>0</v>
@@ -3706,7 +4136,7 @@
         <v>2024A</v>
       </c>
       <c r="B35" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C35" s="1">
         <v>863</v>
@@ -3727,7 +4157,7 @@
         <v>2024B</v>
       </c>
       <c r="B36" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C36" s="1">
         <v>1029</v>
@@ -3748,7 +4178,7 @@
         <v>2024C</v>
       </c>
       <c r="B37" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C37" s="1">
         <v>1240</v>
@@ -3769,7 +4199,7 @@
         <v>2024D</v>
       </c>
       <c r="B38" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C38" s="1">
         <v>1519</v>
@@ -3790,7 +4220,7 @@
         <v>2024E</v>
       </c>
       <c r="B39" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C39" s="1">
         <v>1917</v>

</xml_diff>

<commit_message>
Update footnotes and check numbers - Footnotes updated with latest 2026 plan info - Updated HSA contribution limits - Rechecked cost scenario formulas
</commit_message>
<xml_diff>
--- a/2026 NU health comparison - FAMILY.xlsx
+++ b/2026 NU health comparison - FAMILY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pbh634\Documents\GitHub\nu-health-plan-comparison\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C305C6-DFCD-4145-B4D7-BC671752D787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81BCB715-26E7-4FA8-9C71-8A1802AC2850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{4567C0A1-7649-4947-8B19-B6E9FD1F1145}">
       <text>
         <r>
           <rPr>
@@ -88,7 +88,7 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-NU matches up to $1000 of HSA contributions; this is free money and reduces the yearly cost of care.</t>
+NU matches up to $1000 ($2000 family) of HSA contributions; this is free money and reduces the yearly cost of care.</t>
         </r>
       </text>
     </comment>
@@ -265,7 +265,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="64">
   <si>
     <t>HMO</t>
   </si>
@@ -381,9 +381,6 @@
     <t>Tax savings assumes a reduction in 2026 income taxes due of (2026 Federal tax bracket + 4.95%), where 4.95% is the IL tax rate for 2026.</t>
   </si>
   <si>
-    <t>A FSA tax benefit could be obtained for the PPO plans by contributing to an FSA for the year; however, a FSA is use it or lose it (pre-spending plan) as opposed to a true savings plan.</t>
-  </si>
-  <si>
     <t>% Increase BCBS to UHC</t>
   </si>
   <si>
@@ -456,7 +453,13 @@
     <t>Deductible (1) + OOP costs (1)</t>
   </si>
   <si>
-    <t>This comparison is valid for the "you + spouse" coverage level and assumes individual deductibles within the PPO and HSAe family plans.</t>
+    <t>This comparison is valid for the "you + spouse + children" coverage level and assumes individual deductibles within the PPO and HSAe family plans.</t>
+  </si>
+  <si>
+    <t>In 2026, PPO and HMO plans have a separate prescription drug OOP max. If you will need prescription drug coverage, this increases the expected PPO and HMO costs under the deductible scenarios.</t>
+  </si>
+  <si>
+    <t>A FSA tax benefit could be obtained for the PPO or HMO plans by contributing to an FSA for the year; however, a FSA is use it or lose it (pre-spending plan) as opposed to a true savings plan.</t>
   </si>
 </sst>
 </file>
@@ -709,6 +712,18 @@
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="13" formatCode="0%"/>
     </dxf>
     <dxf>
@@ -759,18 +774,6 @@
         <name val="Calibri"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
@@ -2203,35 +2206,35 @@
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Cap"/>
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Provider"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="PPO" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="HSA+" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="HSAe" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="HMO" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="PPO" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="HSA+" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="HSAe" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="HMO" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="K15:P19" totalsRowShown="0" headerRowDxfId="29" headerRowBorderDxfId="28" tableBorderDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="K15:P19" totalsRowShown="0" headerRowDxfId="33" headerRowBorderDxfId="32" tableBorderDxfId="31">
   <autoFilter ref="K15:P19" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="6">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Cap"/>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Provider" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="PPO" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="HSA+" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="HSAe" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="HMO" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Provider" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="PPO" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="HSA+" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="HSAe" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="HMO" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table5" displayName="Table5" ref="I4:I11" totalsRowShown="0" headerRowDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table5" displayName="Table5" ref="I4:I11" totalsRowShown="0" headerRowDxfId="25">
   <autoFilter ref="I4:I11" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Federal Tax Brackets" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Federal Tax Brackets" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2242,10 +2245,10 @@
   <autoFilter ref="L1:P6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Salary tier"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="PPO" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="HSA+" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="HSAe" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="HMO" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="PPO" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="HSA+" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="HSAe" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="HMO" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2607,10 +2610,10 @@
         <v>34</v>
       </c>
       <c r="C1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" t="s">
         <v>43</v>
-      </c>
-      <c r="D1" t="s">
-        <v>44</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -2631,10 +2634,10 @@
         <v>34</v>
       </c>
       <c r="N1" t="s">
+        <v>42</v>
+      </c>
+      <c r="O1" t="s">
         <v>43</v>
-      </c>
-      <c r="O1" t="s">
-        <v>44</v>
       </c>
       <c r="P1" t="s">
         <v>0</v>
@@ -2642,7 +2645,7 @@
     </row>
     <row r="2" spans="1:16">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2" s="3">
         <f>VLOOKUP($G$2,Table2[#All],COLUMN(),0)</f>
@@ -2687,7 +2690,7 @@
     </row>
     <row r="3" spans="1:16">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3">
@@ -2853,7 +2856,7 @@
         <v>35</v>
       </c>
       <c r="H7" s="17">
-        <v>6550</v>
+        <v>6750</v>
       </c>
       <c r="I7" s="12">
         <v>0.22</v>
@@ -2861,7 +2864,7 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B8" s="5">
         <f>VLOOKUP($H$2,$L$9:$P$10,COLUMN(),0)</f>
@@ -2880,7 +2883,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I8" s="12">
         <v>0.24</v>
@@ -2895,10 +2898,10 @@
         <v>34</v>
       </c>
       <c r="N8" t="s">
+        <v>42</v>
+      </c>
+      <c r="O8" t="s">
         <v>43</v>
-      </c>
-      <c r="O8" t="s">
-        <v>44</v>
       </c>
       <c r="P8" t="s">
         <v>0</v>
@@ -2906,7 +2909,7 @@
     </row>
     <row r="9" spans="1:16">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B9" s="5">
         <f>VLOOKUP($H$2,$L$11:$P$12,COLUMN(),0)</f>
@@ -2928,7 +2931,7 @@
         <v>0.32</v>
       </c>
       <c r="K9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L9" t="s">
         <v>18</v>
@@ -2948,7 +2951,7 @@
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" s="5">
         <f>VLOOKUP($H$2,$L$16:$P$17,COLUMN(),0)</f>
@@ -2970,7 +2973,7 @@
         <v>0.35</v>
       </c>
       <c r="K10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L10" t="s">
         <v>19</v>
@@ -2984,13 +2987,13 @@
       <c r="O10" s="1">
         <v>8000</v>
       </c>
-      <c r="P10" s="1">
-        <v>0</v>
+      <c r="P10" s="1" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="11" spans="1:16">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11" s="5">
         <f>VLOOKUP($H$2,$L$18:$P$19,COLUMN(),0)</f>
@@ -3012,7 +3015,7 @@
         <v>0.37</v>
       </c>
       <c r="K11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L11" t="s">
         <v>18</v>
@@ -3048,7 +3051,7 @@
         <v>HMO</v>
       </c>
       <c r="K12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L12" t="s">
         <v>19</v>
@@ -3093,7 +3096,7 @@
     </row>
     <row r="14" spans="1:16">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B14" s="3">
         <f>SUM(B4:B8)</f>
@@ -3115,14 +3118,14 @@
     </row>
     <row r="15" spans="1:16" ht="15" customHeight="1">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B15" s="3">
         <f>SUM(B4:B7) + MIN(B8*2,B9)</f>
         <v>4848.6120000000001</v>
       </c>
       <c r="C15" s="3">
-        <f>SUM(C4:C7) + MIN(C8*2,C9)</f>
+        <f>SUM(C4:C7) + C9</f>
         <v>3827.8199999999997</v>
       </c>
       <c r="D15" s="3">
@@ -3146,10 +3149,10 @@
         <v>34</v>
       </c>
       <c r="N15" t="s">
+        <v>42</v>
+      </c>
+      <c r="O15" t="s">
         <v>43</v>
-      </c>
-      <c r="O15" t="s">
-        <v>44</v>
       </c>
       <c r="P15" t="s">
         <v>0</v>
@@ -3157,7 +3160,7 @@
     </row>
     <row r="16" spans="1:16">
       <c r="A16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B16" s="3">
         <f>SUM(B4:B7,B10)</f>
@@ -3176,7 +3179,7 @@
         <v>4533.0360000000001</v>
       </c>
       <c r="K16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L16" t="s">
         <v>18</v>
@@ -3196,26 +3199,26 @@
     </row>
     <row r="17" spans="1:16">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B17" s="3">
-        <f>SUM(B4:B7)+MIN(SUM(B8,B10),B11)</f>
+        <f>SUM(B4:B7) + MIN(SUM(B8,B10),B11)</f>
         <v>7098.6120000000001</v>
       </c>
       <c r="C17" s="3">
-        <f>SUM(C4:C7)+MIN(IF(C10&gt;=C9,C10,C9),C11)</f>
+        <f>SUM(C4:C7) + MIN(IF(C10&gt;=C9,C10,C9),C11)</f>
         <v>3827.8199999999997</v>
       </c>
       <c r="D17" s="3">
-        <f>SUM(D4:D7)+MIN(SUM(D8,D10),D11)</f>
+        <f>SUM(D4:D7) + MIN(SUM(D8,D10),D11)</f>
         <v>9968.7520000000004</v>
       </c>
       <c r="E17" s="3">
-        <f>SUM(E4:E7)+MIN(SUM(E8,E10),E11)</f>
+        <f>SUM(E4:E7) + MIN(SUM(E8,E10),E11)</f>
         <v>4533.0360000000001</v>
       </c>
       <c r="K17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L17" t="s">
         <v>19</v>
@@ -3235,28 +3238,28 @@
     </row>
     <row r="18" spans="1:16">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18" s="3">
-        <f>SUM(B4:B7,B11)</f>
+        <f>SUM(B4:B7) + MIN(B10*2,B11)</f>
         <v>9348.612000000001</v>
       </c>
       <c r="C18" s="3">
-        <f>SUM(C4:C7,C11)</f>
+        <f>SUM(C4:C7) + MIN(C10*2,C11)</f>
         <v>7827.82</v>
       </c>
       <c r="D18" s="3">
-        <f>SUM(D4:D7,D11)</f>
+        <f>SUM(D4:D7) + MIN(D10*2,D11)</f>
         <v>12968.752</v>
       </c>
       <c r="E18" s="3">
-        <f>SUM(E4:E7,E11)</f>
+        <f>SUM(E4:E7) + MIN(E10*2,E11)</f>
         <v>6033.0360000000001</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="K18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L18" t="s">
         <v>18</v>
@@ -3280,7 +3283,7 @@
       <c r="D19" s="22"/>
       <c r="E19" s="22"/>
       <c r="K19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L19" t="s">
         <v>19</v>
@@ -3325,7 +3328,7 @@
     </row>
     <row r="21" spans="1:16">
       <c r="A21" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -3342,7 +3345,9 @@
       <c r="E22" s="7"/>
     </row>
     <row r="23" spans="1:16">
-      <c r="A23" s="2"/>
+      <c r="A23" s="2" t="s">
+        <v>63</v>
+      </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
@@ -3350,7 +3355,7 @@
     </row>
     <row r="24" spans="1:16">
       <c r="A24" s="2" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -3376,8 +3381,32 @@
       <c r="E27" s="7"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B19:E19">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B20:E20">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B13:E13">
-    <cfRule type="colorScale" priority="11">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3389,6 +3418,30 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:E14">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E15">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:E16">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -3400,32 +3453,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E15">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B16:E16">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B17:E17">
-    <cfRule type="colorScale" priority="3">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3438,30 +3467,6 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:E18">
     <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B19:E19">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B20:E20">
-    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3490,7 +3495,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="C14 C17" formula="1"/>
+    <ignoredError sqref="C14:C15 C17" formula="1"/>
   </ignoredErrors>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
@@ -3520,7 +3525,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="B1" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C1" s="23"/>
       <c r="D1" s="23"/>
@@ -3539,16 +3544,16 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
         <v>40</v>
-      </c>
-      <c r="D4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -3695,10 +3700,10 @@
         <v>34</v>
       </c>
       <c r="D14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" t="s">
         <v>43</v>
-      </c>
-      <c r="E14" t="s">
-        <v>44</v>
       </c>
       <c r="F14" t="s">
         <v>0</v>
@@ -3818,7 +3823,7 @@
       <c r="E21" s="23"/>
       <c r="F21" s="23"/>
       <c r="I21" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J21" s="23"/>
       <c r="K21" s="23"/>

</xml_diff>